<commit_message>
did all data and unit of analysis section. Started with descriptive statistics
</commit_message>
<xml_diff>
--- a/data/controles_results/dif_medias/controls_vars/difmedias_controles_baselines_fixed_2018_T1_2.xlsx
+++ b/data/controles_results/dif_medias/controls_vars/difmedias_controles_baselines_fixed_2018_T1_2.xlsx
@@ -57,10 +57,10 @@
     <t>N</t>
   </si>
   <si>
-    <t>91</t>
-  </si>
-  <si>
-    <t>90</t>
+    <t>56</t>
+  </si>
+  <si>
+    <t>55</t>
   </si>
   <si>
     <t xml:space="preserve"> (1) </t>
@@ -72,67 +72,67 @@
     <t>Mean/(SE)</t>
   </si>
   <si>
-    <t>6.16e+05</t>
-  </si>
-  <si>
-    <t>(75840.889)</t>
-  </si>
-  <si>
-    <t>501.155</t>
-  </si>
-  <si>
-    <t>(31.953)</t>
-  </si>
-  <si>
-    <t>3.572</t>
-  </si>
-  <si>
-    <t>(0.041)</t>
-  </si>
-  <si>
-    <t>11.560</t>
-  </si>
-  <si>
-    <t>(1.655)</t>
-  </si>
-  <si>
-    <t>88.933</t>
-  </si>
-  <si>
-    <t>(0.420)</t>
-  </si>
-  <si>
-    <t>1.10e+06</t>
-  </si>
-  <si>
-    <t>(50344.269)</t>
-  </si>
-  <si>
-    <t>2.647</t>
-  </si>
-  <si>
-    <t>(0.117)</t>
-  </si>
-  <si>
-    <t>3.571</t>
-  </si>
-  <si>
-    <t>(0.395)</t>
-  </si>
-  <si>
-    <t>34.571</t>
-  </si>
-  <si>
-    <t>(3.049)</t>
-  </si>
-  <si>
-    <t>0.978</t>
-  </si>
-  <si>
-    <t>(0.015)</t>
-  </si>
-  <si>
-    <t>23</t>
+    <t>5.24e+05</t>
+  </si>
+  <si>
+    <t>(80953.804)</t>
+  </si>
+  <si>
+    <t>503.534</t>
+  </si>
+  <si>
+    <t>(38.331)</t>
+  </si>
+  <si>
+    <t>3.714</t>
+  </si>
+  <si>
+    <t>(0.049)</t>
+  </si>
+  <si>
+    <t>6.411</t>
+  </si>
+  <si>
+    <t>(1.336)</t>
+  </si>
+  <si>
+    <t>87.003</t>
+  </si>
+  <si>
+    <t>(0.512)</t>
+  </si>
+  <si>
+    <t>8.97e+05</t>
+  </si>
+  <si>
+    <t>(55836.359)</t>
+  </si>
+  <si>
+    <t>2.162</t>
+  </si>
+  <si>
+    <t>(0.135)</t>
+  </si>
+  <si>
+    <t>2.339</t>
+  </si>
+  <si>
+    <t>(0.404)</t>
+  </si>
+  <si>
+    <t>29.286</t>
+  </si>
+  <si>
+    <t>(4.490)</t>
+  </si>
+  <si>
+    <t>0.929</t>
+  </si>
+  <si>
+    <t>(0.035)</t>
+  </si>
+  <si>
+    <t>60</t>
   </si>
   <si>
     <t xml:space="preserve"> (2) </t>
@@ -141,58 +141,58 @@
     <t>1</t>
   </si>
   <si>
-    <t>6.57e+05</t>
-  </si>
-  <si>
-    <t>(1.32e+05)</t>
-  </si>
-  <si>
-    <t>474.421</t>
-  </si>
-  <si>
-    <t>(75.665)</t>
-  </si>
-  <si>
-    <t>3.258</t>
-  </si>
-  <si>
-    <t>(0.079)</t>
-  </si>
-  <si>
-    <t>35.087</t>
-  </si>
-  <si>
-    <t>(6.038)</t>
-  </si>
-  <si>
-    <t>91.483</t>
-  </si>
-  <si>
-    <t>(0.662)</t>
+    <t>6.98e+05</t>
+  </si>
+  <si>
+    <t>(1.00e+05)</t>
+  </si>
+  <si>
+    <t>482.463</t>
+  </si>
+  <si>
+    <t>(43.823)</t>
+  </si>
+  <si>
+    <t>3.335</t>
+  </si>
+  <si>
+    <t>(0.048)</t>
+  </si>
+  <si>
+    <t>25.000</t>
+  </si>
+  <si>
+    <t>(3.191)</t>
+  </si>
+  <si>
+    <t>91.511</t>
+  </si>
+  <si>
+    <t>(0.367)</t>
   </si>
   <si>
     <t>1.38e+06</t>
   </si>
   <si>
-    <t>(1.00e+05)</t>
-  </si>
-  <si>
-    <t>3.459</t>
-  </si>
-  <si>
-    <t>(0.183)</t>
-  </si>
-  <si>
-    <t>7.391</t>
-  </si>
-  <si>
-    <t>(0.857)</t>
-  </si>
-  <si>
-    <t>49.826</t>
-  </si>
-  <si>
-    <t>(4.839)</t>
+    <t>(57218.217)</t>
+  </si>
+  <si>
+    <t>3.352</t>
+  </si>
+  <si>
+    <t>(0.119)</t>
+  </si>
+  <si>
+    <t>6.067</t>
+  </si>
+  <si>
+    <t>(0.544)</t>
+  </si>
+  <si>
+    <t>44.200</t>
+  </si>
+  <si>
+    <t>(2.738)</t>
   </si>
   <si>
     <t>1.000</t>
@@ -201,10 +201,10 @@
     <t>(0.000)</t>
   </si>
   <si>
-    <t>114</t>
-  </si>
-  <si>
-    <t>113</t>
+    <t>116</t>
+  </si>
+  <si>
+    <t>115</t>
   </si>
   <si>
     <t>(2)-(1)</t>
@@ -216,34 +216,34 @@
     <t>Mean difference</t>
   </si>
   <si>
-    <t>41250.355</t>
-  </si>
-  <si>
-    <t>-26.735</t>
-  </si>
-  <si>
-    <t>-0.314***</t>
-  </si>
-  <si>
-    <t>23.527***</t>
-  </si>
-  <si>
-    <t>2.551***</t>
-  </si>
-  <si>
-    <t>2.78e+05**</t>
-  </si>
-  <si>
-    <t>0.812***</t>
-  </si>
-  <si>
-    <t>3.820***</t>
-  </si>
-  <si>
-    <t>15.255**</t>
-  </si>
-  <si>
-    <t>0.022</t>
+    <t>1.74e+05</t>
+  </si>
+  <si>
+    <t>-21.071</t>
+  </si>
+  <si>
+    <t>-0.380***</t>
+  </si>
+  <si>
+    <t>18.589***</t>
+  </si>
+  <si>
+    <t>4.508***</t>
+  </si>
+  <si>
+    <t>4.82e+05***</t>
+  </si>
+  <si>
+    <t>1.190***</t>
+  </si>
+  <si>
+    <t>3.727***</t>
+  </si>
+  <si>
+    <t>14.914***</t>
+  </si>
+  <si>
+    <t>0.071**</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
finished creating the proper tables and got all the other type of crimes
</commit_message>
<xml_diff>
--- a/data/controles_results/dif_medias/controls_vars/difmedias_controles_baselines_fixed_2018_T1_2.xlsx
+++ b/data/controles_results/dif_medias/controls_vars/difmedias_controles_baselines_fixed_2018_T1_2.xlsx
@@ -57,10 +57,10 @@
     <t>N</t>
   </si>
   <si>
-    <t>56</t>
-  </si>
-  <si>
-    <t>55</t>
+    <t>91</t>
+  </si>
+  <si>
+    <t>90</t>
   </si>
   <si>
     <t xml:space="preserve"> (1) </t>
@@ -72,67 +72,67 @@
     <t>Mean/(SE)</t>
   </si>
   <si>
-    <t>5.24e+05</t>
-  </si>
-  <si>
-    <t>(80953.804)</t>
-  </si>
-  <si>
-    <t>503.534</t>
-  </si>
-  <si>
-    <t>(38.331)</t>
-  </si>
-  <si>
-    <t>3.714</t>
-  </si>
-  <si>
-    <t>(0.049)</t>
-  </si>
-  <si>
-    <t>6.411</t>
-  </si>
-  <si>
-    <t>(1.336)</t>
-  </si>
-  <si>
-    <t>87.003</t>
-  </si>
-  <si>
-    <t>(0.512)</t>
-  </si>
-  <si>
-    <t>8.97e+05</t>
-  </si>
-  <si>
-    <t>(55836.359)</t>
-  </si>
-  <si>
-    <t>2.162</t>
-  </si>
-  <si>
-    <t>(0.135)</t>
-  </si>
-  <si>
-    <t>2.339</t>
-  </si>
-  <si>
-    <t>(0.404)</t>
-  </si>
-  <si>
-    <t>29.286</t>
-  </si>
-  <si>
-    <t>(4.490)</t>
-  </si>
-  <si>
-    <t>0.929</t>
-  </si>
-  <si>
-    <t>(0.035)</t>
-  </si>
-  <si>
-    <t>60</t>
+    <t>6.16e+05</t>
+  </si>
+  <si>
+    <t>(75840.889)</t>
+  </si>
+  <si>
+    <t>501.155</t>
+  </si>
+  <si>
+    <t>(31.953)</t>
+  </si>
+  <si>
+    <t>3.572</t>
+  </si>
+  <si>
+    <t>(0.041)</t>
+  </si>
+  <si>
+    <t>11.560</t>
+  </si>
+  <si>
+    <t>(1.655)</t>
+  </si>
+  <si>
+    <t>88.933</t>
+  </si>
+  <si>
+    <t>(0.420)</t>
+  </si>
+  <si>
+    <t>1.10e+06</t>
+  </si>
+  <si>
+    <t>(50344.269)</t>
+  </si>
+  <si>
+    <t>2.647</t>
+  </si>
+  <si>
+    <t>(0.117)</t>
+  </si>
+  <si>
+    <t>3.571</t>
+  </si>
+  <si>
+    <t>(0.395)</t>
+  </si>
+  <si>
+    <t>34.571</t>
+  </si>
+  <si>
+    <t>(3.049)</t>
+  </si>
+  <si>
+    <t>0.978</t>
+  </si>
+  <si>
+    <t>(0.015)</t>
+  </si>
+  <si>
+    <t>23</t>
   </si>
   <si>
     <t xml:space="preserve"> (2) </t>
@@ -141,58 +141,58 @@
     <t>1</t>
   </si>
   <si>
-    <t>6.98e+05</t>
+    <t>6.57e+05</t>
+  </si>
+  <si>
+    <t>(1.32e+05)</t>
+  </si>
+  <si>
+    <t>474.421</t>
+  </si>
+  <si>
+    <t>(75.665)</t>
+  </si>
+  <si>
+    <t>3.258</t>
+  </si>
+  <si>
+    <t>(0.079)</t>
+  </si>
+  <si>
+    <t>35.087</t>
+  </si>
+  <si>
+    <t>(6.038)</t>
+  </si>
+  <si>
+    <t>91.483</t>
+  </si>
+  <si>
+    <t>(0.662)</t>
+  </si>
+  <si>
+    <t>1.38e+06</t>
   </si>
   <si>
     <t>(1.00e+05)</t>
   </si>
   <si>
-    <t>482.463</t>
-  </si>
-  <si>
-    <t>(43.823)</t>
-  </si>
-  <si>
-    <t>3.335</t>
-  </si>
-  <si>
-    <t>(0.048)</t>
-  </si>
-  <si>
-    <t>25.000</t>
-  </si>
-  <si>
-    <t>(3.191)</t>
-  </si>
-  <si>
-    <t>91.511</t>
-  </si>
-  <si>
-    <t>(0.367)</t>
-  </si>
-  <si>
-    <t>1.38e+06</t>
-  </si>
-  <si>
-    <t>(57218.217)</t>
-  </si>
-  <si>
-    <t>3.352</t>
-  </si>
-  <si>
-    <t>(0.119)</t>
-  </si>
-  <si>
-    <t>6.067</t>
-  </si>
-  <si>
-    <t>(0.544)</t>
-  </si>
-  <si>
-    <t>44.200</t>
-  </si>
-  <si>
-    <t>(2.738)</t>
+    <t>3.459</t>
+  </si>
+  <si>
+    <t>(0.183)</t>
+  </si>
+  <si>
+    <t>7.391</t>
+  </si>
+  <si>
+    <t>(0.857)</t>
+  </si>
+  <si>
+    <t>49.826</t>
+  </si>
+  <si>
+    <t>(4.839)</t>
   </si>
   <si>
     <t>1.000</t>
@@ -201,10 +201,10 @@
     <t>(0.000)</t>
   </si>
   <si>
-    <t>116</t>
-  </si>
-  <si>
-    <t>115</t>
+    <t>114</t>
+  </si>
+  <si>
+    <t>113</t>
   </si>
   <si>
     <t>(2)-(1)</t>
@@ -216,34 +216,34 @@
     <t>Mean difference</t>
   </si>
   <si>
-    <t>1.74e+05</t>
-  </si>
-  <si>
-    <t>-21.071</t>
-  </si>
-  <si>
-    <t>-0.380***</t>
-  </si>
-  <si>
-    <t>18.589***</t>
-  </si>
-  <si>
-    <t>4.508***</t>
-  </si>
-  <si>
-    <t>4.82e+05***</t>
-  </si>
-  <si>
-    <t>1.190***</t>
-  </si>
-  <si>
-    <t>3.727***</t>
-  </si>
-  <si>
-    <t>14.914***</t>
-  </si>
-  <si>
-    <t>0.071**</t>
+    <t>41250.355</t>
+  </si>
+  <si>
+    <t>-26.735</t>
+  </si>
+  <si>
+    <t>-0.314***</t>
+  </si>
+  <si>
+    <t>23.527***</t>
+  </si>
+  <si>
+    <t>2.551***</t>
+  </si>
+  <si>
+    <t>2.78e+05**</t>
+  </si>
+  <si>
+    <t>0.812***</t>
+  </si>
+  <si>
+    <t>3.820***</t>
+  </si>
+  <si>
+    <t>15.255**</t>
+  </si>
+  <si>
+    <t>0.022</t>
   </si>
 </sst>
 </file>

</xml_diff>